<commit_message>
Add SSI shared header/footer partials; refactor find-your-beans quiz
Introduce /partials/header.html and footer.html included via Apache SSI
(AddOutputFilter INCLUDES .html), with an ssi-test/ proof page; disallow
/partials/ in robots.txt. Make quiz option data-vals unique slugs with a
brew-family mapping layer so milk/brew/budget matching stays correct.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/THE-BEANS-HUB-PAGES-AND-FUNNEL.xlsx
+++ b/THE-BEANS-HUB-PAGES-AND-FUNNEL.xlsx
@@ -5164,7 +5164,7 @@
       </c>
       <c r="F5" s="42" t="inlineStr">
         <is>
-          <t>black</t>
+          <t>black-no-milk</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="F6" s="42" t="inlineStr">
         <is>
-          <t>milk</t>
+          <t>with-milk</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="F7" s="42" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>a-bit-of-both</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="F8" s="42" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>still-figuring-it-out</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="F9" s="42" t="inlineStr">
         <is>
-          <t>espresso</t>
+          <t>espresso-machine</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="F10" s="42" t="inlineStr">
         <is>
-          <t>espresso</t>
+          <t>moka-pot</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
-          <t>filter</t>
+          <t>v60-pour-over</t>
         </is>
       </c>
     </row>
@@ -5292,7 +5292,7 @@
       </c>
       <c r="F12" s="42" t="inlineStr">
         <is>
-          <t>filter</t>
+          <t>french-press</t>
         </is>
       </c>
     </row>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="F13" s="42" t="inlineStr">
         <is>
-          <t>filter</t>
+          <t>aeropress</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F14" s="42" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>im-just-starting-out</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5578,7 @@
       </c>
       <c r="F27" s="42" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>under-rm30</t>
         </is>
       </c>
     </row>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="F28" s="42" t="inlineStr">
         <is>
-          <t>everyday</t>
+          <t>rm30-49</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="F29" s="42" t="inlineStr">
         <is>
-          <t>premium</t>
+          <t>rm50-79</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="F30" s="42" t="inlineStr">
         <is>
-          <t>splurge</t>
+          <t>rm80-plus</t>
         </is>
       </c>
     </row>
@@ -5642,7 +5642,7 @@
       </c>
       <c r="F31" s="42" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>price-isnt-the-deciding-factor</t>
         </is>
       </c>
     </row>

</xml_diff>